<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.001-06 Victorino et le galet lisse
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-06.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-06.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bord de rivière</t>
+          <t>bord de rivière, nappe, galet, cailloux, panier, pain, herbe, eau, soleil</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Près de l'eau, Victorino trouve un galet lisse. Il dit sa joie. Il le fait toucher à papa et maman.</t>
+          <t>Le panier craque contre l'herbe. Sur le bord, un éclat de berge luit. Victorino veut le galet, maintenant. Trop lisse : il glisse, tombe. Poitrine trop vite. Sourire parti. Papa s'accroupit. Je suis content. Merci vécu. Deuxième ruse : le galet glisse vers l'eau. Il refuse de foncer. Il fait toucher. Un éclat de berge tient près du bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>L'eau fait tic, tic, tic. Elle tape les cailloux. Le chemin est chaud. Les cigales chantent loin. Le soleil pique un peu le nez. Des cailloux blancs brillent. Une nappe est posée dans l'herbe. Le vent bouge un coin. Papa pose le panier. Le pain sent encore chaud. Maman tient la main de Victorino. On reste près de l'eau. Les pieds sur l'herbe, d'accord ? D'accord, papa. En ce moment, Victorino regarde le bord. L'eau brille. Elle est claire. Un brin d'herbe tremble. Un galet gris attend dans l'herbe sèche. Il est lisse. Il est tiède. Un galet ! Tu peux le prendre. Victorino le prend dans les deux mains. Le galet est chaud du soleil. Parce qu'il a trouvé le galet. Ses joues sont chaudes. Son ventre est léger. Un sourire arrive. Je suis content. C'est de la joie. Bravo, Victorino. Tu as dit ta joie. On peut partager ? Oui. On touche ensemble. Victorino tend le galet. Papa le touche. Maman le touche. Il est lisse, hein ? Oui. Lisse. Merci. Tu nous invites. Je suis content. Tu as de la joie ? Oui, papa. L'eau continue tic, tic, tic. Un oiseau passe très bas. Le galet reste dans sa main.</t>
+          <t>Le panier craque contre l'herbe. Tu poses le pain, maman ? Oui, sur la nappe. Un coin de nappe se lève. Il vole, papa ! Le vent le pousse. Le pain sent le soleil. Ça sent bon. Tu le sens, Victorino ? Oui, maman. L'eau de la rivière fait tic. Ça tape les cailloux, au bord. Tu entends le tic ? Oui, le tic. Le chemin brûle un peu les pieds. Il est chaud ! On reste dans l'herbe ? Oui, papa. Les cigales chantent, très loin. Le soleil pique un peu le nez. Il pique, maman. Le nez est tiède ? Un peu. Maman s'assoit près du panier. Ça chauffe les genoux. Les genoux sont bien ? Oui, papa. Un éclat de berge luit. Il brille, papa ! Tu le vois, près du bord ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. Il allume l'herbe. Un galet gris attend dans l'herbe. Un galet ! Il est lisse, Victorino ? Je le prends ! En ce moment, Victorino veut le galet. Je le veux, maintenant ! Tout de suite ? Oui, papa. Les deux mains serrent trop vite. Le galet est trop lisse. Il glisse ! Le galet tombe dans l'herbe sèche. Ça fait un bruit mou. Oh. Victorino reste les mains ouvertes. Sa poitrine va trop vite. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le galet, Victorino ? Il est là. Tes mains sont chaudes ? Un peu, maman. Victorino cherche dans l'herbe. Le galet est tiède, sous les doigts. Je le tiens. Un sourire revient, tout petit. Je suis content. Tu le serres, Victorino ? Oui. Il chauffe la paume ? Oui, maman. L'éclat de berge tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>L'eau fait tic, tic, tic. Elle tape les cailloux. Le chemin est chaud. Les cigales chantent loin. Le soleil pique un peu le nez. Des cailloux blancs brillent. Une nappe est posée dans l'herbe. Le vent bouge un coin. Papa pose le panier. Le pain sent encore chaud. Maman tient la main de Victorino. On reste près de l'eau. Les pieds sur l'herbe, d'accord ? D'accord, papa. En ce moment, Victorino regarde le bord. L'eau brille. Elle est claire. Un brin d'herbe tremble. Un galet gris attend dans l'herbe sèche. Il est lisse. Il est tiède. Un galet ! Tu peux le prendre. Victorino le prend dans les deux mains. Le galet est chaud du soleil. Parce qu'il a trouvé le galet. Ses joues sont chaudes. Son ventre est léger. Un sourire arrive. Je suis content. C'est de la joie. Bravo, Victorino. Tu as dit ta joie. On peut partager ? Oui. On touche ensemble. Victorino tend le galet. Papa le touche. Maman le touche. Il est lisse, hein ? Oui. Lisse. Merci. Tu nous invites. Je suis content. Tu as de la joie ? Oui, papa. L'eau continue tic, tic, tic. Un oiseau passe très bas. Le galet reste dans sa main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le panier craque contre l'herbe. Tu poses le pain, maman ? Oui, sur la nappe. Un coin de nappe se lève. Il vole, papa ! Le vent le pousse. Le pain sent le soleil. Ça sent bon. Tu le sens, Victorino ? Oui, maman. L'eau de la rivière fait tic. Ça tape les cailloux, au bord. Tu entends le tic ? Oui, le tic. Le chemin brûle un peu les pieds. Il est chaud ! On reste dans l'herbe ? Oui, papa. Les cigales chantent, très loin. Le soleil pique un peu le nez. Il pique, maman. Le nez est tiède ? Un peu. Maman s'assoit près du panier. Ça chauffe les genoux. Les genoux sont bien ? Oui, papa. Un &lt;emphasis level="moderate"&gt;éclat de berge&lt;/emphasis&gt; luit. Il brille, papa ! Tu le vois, près du bord ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. Il allume l'herbe. Un galet gris attend dans l'herbe. Un galet ! Il est lisse, Victorino ? Je le prends ! En ce moment, Victorino veut le galet. Je le veux, maintenant ! Tout de suite ? Oui, papa. Les deux mains serrent trop vite. Le galet est trop lisse. Il glisse ! Le galet tombe dans l'herbe sèche. Ça fait un bruit mou. Oh. Victorino reste les mains ouvertes. Sa poitrine va trop vite. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le galet, Victorino ? Il est là. Tes mains sont chaudes ? Un peu, maman. Victorino cherche dans l'herbe. Le galet est tiède, sous les doigts. Je le tiens. Un sourire revient, tout petit. Je suis content. Tu le serres, Victorino ? Oui. Il chauffe la paume ? Oui, maman. L'éclat de berge tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Eva marche au bord de l'eau. Maman tient sa main. Papa ramasse du bois. Eva trouve un galet lisse. Il est gris et chaud. Eva sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Eva dit : je suis &lt;emphasis&gt;content&lt;/emphasis&gt;e. Papa dit : c'est de la joie. Eva tend le galet. Elle dit : on peut partager. Papa touche le galet. Maman touche le galet. Ils sourient ensemble. Eva dit encore : je suis contente. La joie est là, près de l'eau. Le galet reste dans sa poche.&lt;/slow&gt; [pause]</t>
+          <t>Le panier craque contre l'herbe. Tu poses le pain, maman ? Oui, sur la nappe. Un coin de nappe se lève. Il vole, papa ! Le vent le pousse. Le pain sent le soleil. Ça sent bon. Tu le sens, Victorino ? Oui, maman. L'eau de la rivière fait tic. Ça tape les cailloux, au bord. Tu entends le tic ? Oui, le tic. Le chemin brûle un peu les pieds. Il est chaud ! On reste dans l'herbe ? Oui, papa. Les cigales chantent, très loin. Le soleil pique un peu le nez. Il pique, maman. Le nez est tiède ? Un peu. Maman s'assoit près du panier. Ça chauffe les genoux. Les genoux sont bien ? Oui, papa. Un &lt;emphasis&gt;éclat de berge&lt;/emphasis&gt; luit. Il brille, papa ! Tu le vois, près du bord ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. Il allume l'herbe. Un galet gris attend dans l'herbe. Un galet ! Il est lisse, Victorino ? Je le prends ! En ce moment, Victorino veut le galet. Je le veux, maintenant ! Tout de suite ? Oui, papa. Les deux mains serrent trop vite. Le galet est trop lisse. Il glisse ! Le galet tombe dans l'herbe sèche. Ça fait un bruit mou. Oh. Victorino reste les mains ouvertes. Sa poitrine va trop vite. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le galet, Victorino ? Il est là. Tes mains sont chaudes ? Un peu, maman. Victorino cherche dans l'herbe. Le galet est tiède, sous les doigts. Je le tiens. Un sourire revient, tout petit. Je suis content. Tu le serres, Victorino ? Oui. Il chauffe la paume ? Oui, maman. L'éclat de berge tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>éclat de berge</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,56 +1319,84 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_galet_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|L'eau fait tic, tic, tic.
-narrateur|Elle tape les cailloux.
-narrateur|Le chemin est chaud.
-narrateur|Les cigales chantent loin.
+          <t>narrateur|Le panier craque contre l'herbe.
+papa|Tu poses le pain, maman ?
+maman|Oui, sur la nappe.
+narrateur|Un coin de nappe se lève.
+enfant-m|Il vole, papa !
+papa|Le vent le pousse.
+narrateur|Le pain sent le soleil.
+enfant-m|Ça sent bon.
+maman|Tu le sens, Victorino ?
+enfant-m|Oui, maman.
+narrateur|L'eau de la rivière fait tic.
+narrateur|Ça tape les cailloux, au bord.
+maman|Tu entends le tic ?
+enfant-m|Oui, le tic.
+narrateur|Le chemin brûle un peu les pieds.
+enfant-m|Il est chaud !
+papa|On reste dans l'herbe ?
+enfant-m|Oui, papa.
+narrateur|Les cigales chantent, très loin.
 narrateur|Le soleil pique un peu le nez.
-narrateur|Des cailloux blancs brillent.
-narrateur|Une nappe est posée dans l'herbe.
-narrateur|Le vent bouge un coin.
-narrateur|Papa pose le panier.
-narrateur|Le pain sent encore chaud.
-narrateur|Maman tient la main de Victorino.
-maman|On reste près de l'eau.
-papa|Les pieds sur l'herbe, d'accord ?
-enfant-m|D'accord, papa.
-narrateur|En ce moment, Victorino regarde le bord.
-narrateur|L'eau brille. Elle est claire.
-narrateur|Un brin d'herbe tremble.
-narrateur|Un galet gris attend dans l'herbe sèche.
-narrateur|Il est lisse. Il est tiède.
+enfant-m|Il pique, maman.
+maman|Le nez est tiède ?
+enfant-m|Un peu.
+narrateur|Maman s'assoit près du panier.
+enfant-m|Ça chauffe les genoux.
+papa|Les genoux sont bien ?
+enfant-m|Oui, papa.
+narrateur|Un éclat de berge luit.
+enfant-m|Il brille, papa !
+papa|Tu le vois, près du bord ?
+enfant-m|Oui, un petit point.
+maman|Le soleil le touche.
+narrateur|Un rayon glisse sur le bord.
+enfant-m|Il allume l'herbe.
+narrateur|Un galet gris attend dans l'herbe.
 enfant-m|Un galet !
-maman|Tu peux le prendre.
-narrateur|Victorino le prend dans les deux mains.
-narrateur|Le galet est chaud du soleil.
-narrateur|Parce qu'il a trouvé le galet.
-narrateur|Ses joues sont chaudes.
-narrateur|Son ventre est léger.
-narrateur|Un sourire arrive.
+maman|Il est lisse, Victorino ?
+enfant-m|Je le prends !
+narrateur|En ce moment, Victorino veut le galet.
+enfant-m|Je le veux, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Les deux mains serrent trop vite.
+narrateur|Le galet est trop lisse.
+enfant-m|Il glisse !
+narrateur|Le galet tombe dans l'herbe sèche.
+narrateur|Ça fait un bruit mou.
+enfant-m|Oh.
+narrateur|Victorino reste les mains ouvertes.
+narrateur|Sa poitrine va trop vite.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois le galet, Victorino ?
+enfant-m|Il est là.
+maman|Tes mains sont chaudes ?
+enfant-m|Un peu, maman.
+narrateur|Victorino cherche dans l'herbe.
+narrateur|Le galet est tiède, sous les doigts.
+enfant-m|Je le tiens.
+narrateur|Un sourire revient, tout petit.
 enfant-m|Je suis content.
-papa|C'est de la joie.
-maman|Bravo, Victorino.
-maman|Tu as dit ta joie.
-enfant-m|On peut partager ?
-papa|Oui. On touche ensemble.
-narrateur|Victorino tend le galet.
-narrateur|Papa le touche.
-narrateur|Maman le touche.
-papa|Il est lisse, hein ?
-enfant-m|Oui. Lisse.
-maman|Merci. Tu nous invites.
-enfant-m|Je suis content.
-papa|Tu as de la joie ?
-enfant-m|Oui, papa.
-narrateur|L'eau continue tic, tic, tic.
-narrateur|Un oiseau passe très bas.
-narrateur|Le galet reste dans sa main.</t>
+papa|Tu le serres, Victorino ?
+enfant-m|Oui.
+maman|Il chauffe la paume ?
+enfant-m|Oui, maman.
+narrateur|L'éclat de berge tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1405,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino sourit. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Victorino&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Eva sourit. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Victorino&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1435,7 +1463,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Eva sent de la joie. Que dit-elle ?</t>
+          <t>Victorino sent de la joie. Que dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1473,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1484,7 +1512,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1499,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Victorino</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1541,7 +1573,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1551,12 +1583,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=victorino_sourit_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorino sourit. Que dit-il ?</t>
+          <t>narrateur|Victorino sourit.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1583,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino serre encore le galet. C'est de la joie. Oui. Tu es content. Tu as partagé. Tu as fini de le montrer ? Oui. Victorino essuie ses mains. Le galet est propre et chaud.</t>
+          <t>Victorino veut montrer le galet. Vous touchez, maintenant ! Les mots se bousculent dans sa bouche. Trop vite. Victorino avance les mains, trop vite. Le galet penche vers l'herbe. Puis il s'arrête. Il referme les doigts, puis ouvre. Personne ne parle. Il observe le galet, un instant. Il écoute l'eau, près du bord. Tu touches, papa ? Je touche, Victorino ? Oui. Papa pose un doigt sur le galet. Toi aussi, maman. J'approche le doigt ? Oui, maman. Maman touche le galet, tout près. Il est lisse, hein ? Oui. Lisse. Merci, Victorino. Papa reste à la même hauteur. Il chauffe sous le doigt ? Un peu. Le ventre de Victorino se desserre. Les épaules se relèvent un peu. On reste près du galet ? Oui. Je suis content. Tes genoux sont au chaud ? Un peu, maman. Le galet reste dans les deux mains. Il est tiède. Tu le vois, le galet ? Oui, papa. La nappe attend, Victorino ? Après. Un rayon passe sur le bord. Il allume le galet. On tient ensemble ? Oui. Les cailloux font tic, au bord. Je les entends. Le pain reste dans le panier ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorino serre encore le galet. C'est de la joie. Oui. Tu es content. Tu as partagé. Tu as fini de le montrer ? Oui. Victorino essuie ses mains. Le galet est propre et chaud.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino veut montrer le galet. Vous touchez, maintenant ! Les mots se bousculent dans sa bouche. Trop vite. Victorino avance les mains, trop vite. Le galet penche vers l'herbe. Puis il s'arrête. Il referme les doigts, puis ouvre. Personne ne parle. Il observe le galet, un instant. Il écoute l'eau, près du bord. Tu touches, papa ? Je touche, Victorino ? Oui. Papa pose un doigt sur le galet. Toi aussi, maman. J'approche le doigt ? Oui, maman. Maman touche le galet, tout près. Il est lisse, hein ? Oui. Lisse. Merci, Victorino. Papa reste à la même hauteur. Il chauffe sous le doigt ? Un peu. Le ventre de Victorino se desserre. Les épaules se relèvent un peu. On reste près du galet ? Oui. Je suis &lt;emphasis level="moderate"&gt;content&lt;/emphasis&gt;. Tes genoux sont au chaud ? Un peu, maman. Le galet reste dans les deux mains. Il est tiède. Tu le vois, le galet ? Oui, papa. La nappe attend, Victorino ? Après. Un rayon passe sur le bord. Il allume le galet. On tient ensemble ? Oui. Les cailloux font tic, au bord. Je les entends. Le pain reste dans le panier ? Oui, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Eva a nommé sa joie. Elle a partagé avec papa et maman. Être &lt;emphasis&gt;content&lt;/emphasis&gt;, c'est bien.&lt;/slow&gt; [pause]</t>
+          <t>Victorino veut montrer le galet. Vous touchez, maintenant ! Les mots se bousculent dans sa bouche. Trop vite. Victorino avance les mains, trop vite. Le galet penche vers l'herbe. Puis il s'arrête. Il referme les doigts, puis ouvre. Personne ne parle. Il observe le galet, un instant. Il écoute l'eau, près du bord. Tu touches, papa ? Je touche, Victorino ? Oui. Papa pose un doigt sur le galet. Toi aussi, maman. J'approche le doigt ? Oui, maman. Maman touche le galet, tout près. Il est lisse, hein ? Oui. Lisse. Merci, Victorino. Papa reste à la même hauteur. Il chauffe sous le doigt ? Un peu. Le ventre de Victorino se desserre. Les épaules se relèvent un peu. On reste près du galet ? Oui. Je suis &lt;emphasis&gt;content&lt;/emphasis&gt;. Tes genoux sont au chaud ? Un peu, maman. Le galet reste dans les deux mains. Il est tiède. Tu le vois, le galet ? Oui, papa. La nappe attend, Victorino ? Après. Un rayon passe sur le bord. Il allume le galet. On tient ensemble ? Oui. Les cailloux font tic, au bord. Je les entends. Le pain reste dans le panier ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1640,18 +1673,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1681,23 +1714,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1706,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1718,23 +1751,62 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_fait_toucher_le_galet; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorino serre encore le galet.
-enfant-m|C'est de la joie.
-maman|Oui. Tu es content.
-maman|Tu as partagé.
-papa|Tu as fini de le montrer ?
+          <t>narrateur|Victorino veut montrer le galet.
+enfant-m|Vous touchez, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Trop vite.
+narrateur|Victorino avance les mains, trop vite.
+narrateur|Le galet penche vers l'herbe.
+narrateur|Puis il s'arrête.
+narrateur|Il referme les doigts, puis ouvre.
+narrateur|Personne ne parle.
+narrateur|Il observe le galet, un instant.
+narrateur|Il écoute l'eau, près du bord.
+enfant-m|Tu touches, papa ?
+papa|Je touche, Victorino ?
 enfant-m|Oui.
-narrateur|Victorino essuie ses mains.
-narrateur|Le galet est propre et chaud.</t>
+narrateur|Papa pose un doigt sur le galet.
+enfant-m|Toi aussi, maman.
+maman|J'approche le doigt ?
+enfant-m|Oui, maman.
+narrateur|Maman touche le galet, tout près.
+papa|Il est lisse, hein ?
+enfant-m|Oui.
+enfant-m|Lisse.
+papa|Merci, Victorino.
+narrateur|Papa reste à la même hauteur.
+maman|Il chauffe sous le doigt ?
+enfant-m|Un peu.
+narrateur|Le ventre de Victorino se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du galet ?
+enfant-m|Oui.
+enfant-m|Je suis content.
+maman|Tes genoux sont au chaud ?
+enfant-m|Un peu, maman.
+narrateur|Le galet reste dans les deux mains.
+enfant-m|Il est tiède.
+papa|Tu le vois, le galet ?
+enfant-m|Oui, papa.
+maman|La nappe attend, Victorino ?
+enfant-m|Après.
+narrateur|Un rayon passe sur le bord.
+enfant-m|Il allume le galet.
+papa|On tient ensemble ?
+enfant-m|Oui.
+narrateur|Les cailloux font tic, au bord.
+enfant-m|Je les entends.
+maman|Le pain reste dans le panier ?
+enfant-m|Oui, maman.</t>
         </is>
       </c>
     </row>
@@ -1761,17 +1833,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Victorino glisse le galet dans sa poche. La poche fait un petit poids. On va à la nappe ? Oui, maman. Tu as bien invité. Je suis content. La joie est là, près de l'eau. Ils s'assoient sur la nappe. Tu as les pieds dans l'herbe ? Oui. Dans l'herbe. Le pain attend dans le panier. L'eau chante encore. On goûte le pain après ? Après. Le galet d'abord.</t>
+          <t>Maman tire un coin de nappe. Le panier est un peu lourd. Le galet, maintenant ! Victorino serre trop fort, tout de suite. Le galet glisse de sa main. Il glisse ! Le galet roule vers l'eau. Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le galet, un instant. Il écoute l'eau, près des cailloux. Sur le bord, un éclat de berge luit. Là, sur le bord. Victorino pose deux doigts, sans se presser. Le galet s'arrête, trop lisse. On tient le galet ? Oui, papa. Papa pose un doigt, avec lui. Maman pose un doigt, aussi. Vous touchez. Il est froid, près de l'eau ? Un peu. Le galet sent l'herbe tiède. Une petite trace d'eau reste. Poumf. Le galet tient, Victorino ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. La nappe reste ouverte, près d'eux. Elle sent le pain. On reste ici, Victorino ? Oui. Les cailloux font tic, au bord. Le tic est là. Tu le serres sans forcer ? Oui, maman. On touche ensemble ? Oui. Trois doigts tiennent le galet. Il ne part plus.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Victorino glisse le galet dans sa poche. La poche fait un petit poids. On va à la nappe ? Oui, maman. Tu as bien invité. Je suis content. La joie est là, près de l'eau. Ils s'assoient sur la nappe. Tu as les pieds dans l'herbe ? Oui. Dans l'herbe. Le pain attend dans le panier. L'eau chante encore. On goûte le pain après ? Après. Le galet d'abord.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman tire un coin de nappe. Le panier est un peu lourd. Le galet, maintenant ! Victorino serre trop fort, tout de suite. Le galet glisse de sa main. Il glisse ! Le galet roule vers l'eau. Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le galet, un instant. Il écoute l'eau, près des cailloux. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de berge&lt;/emphasis&gt; luit. Là, sur le bord. Victorino pose deux doigts, sans se presser. Le galet s'arrête, trop lisse. On tient le galet ? Oui, papa. Papa pose un doigt, avec lui. Maman pose un doigt, aussi. Vous touchez. Il est froid, près de l'eau ? Un peu. Le galet sent l'herbe tiède. Une petite trace d'eau reste. Poumf. Le galet tient, Victorino ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. La nappe reste ouverte, près d'eux. Elle sent le pain. On reste ici, Victorino ? Oui. Les cailloux font tic, au bord. Le tic est là. Tu le serres sans forcer ? Oui, maman. On touche ensemble ? Oui. Trois doigts tiennent le galet. Il ne part plus.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Eva essuie ses &lt;emphasis&gt;main&lt;/emphasis&gt;s. L'eau chante. Papa lui prend la main.&lt;/slow&gt; [pause]</t>
+          <t>Maman tire un coin de nappe. Le panier est un peu lourd. Le galet, maintenant ! Victorino serre trop fort, tout de suite. Le galet glisse de sa main. Il glisse ! Le galet roule vers l'eau. Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le galet, un instant. Il écoute l'eau, près des cailloux. Sur le bord, un &lt;emphasis&gt;éclat de berge&lt;/emphasis&gt; luit. Là, sur le bord. Victorino pose deux doigts, sans se presser. Le galet s'arrête, trop lisse. On tient le galet ? Oui, papa. Papa pose un doigt, avec lui. Maman pose un doigt, aussi. Vous touchez. Il est froid, près de l'eau ? Un peu. Le galet sent l'herbe tiède. Une petite trace d'eau reste. Poumf. Le galet tient, Victorino ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. La nappe reste ouverte, près d'eux. Elle sent le pain. On reste ici, Victorino ? Oui. Les cailloux font tic, au bord. Le tic est là. Tu le serres sans forcer ? Oui, maman. On touche ensemble ? Oui. Trois doigts tiennent le galet. Il ne part plus. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1818,18 +1890,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1852,30 +1924,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de berge</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1884,10 +1956,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1896,25 +1968,64 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_galet_glisse_vers_leau_il_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Victorino glisse le galet dans sa poche.
-narrateur|La poche fait un petit poids.
-maman|On va à la nappe ?
+          <t>narrateur|Maman tire un coin de nappe.
+narrateur|Le panier est un peu lourd.
+enfant-m|Le galet, maintenant !
+narrateur|Victorino serre trop fort, tout de suite.
+narrateur|Le galet glisse de sa main.
+enfant-m|Il glisse !
+narrateur|Le galet roule vers l'eau.
+narrateur|Victorino avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Victorino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le galet, un instant.
+narrateur|Il écoute l'eau, près des cailloux.
+narrateur|Sur le bord, un éclat de berge luit.
+enfant-m|Là, sur le bord.
+narrateur|Victorino pose deux doigts, sans se presser.
+narrateur|Le galet s'arrête, trop lisse.
+papa|On tient le galet ?
+enfant-m|Oui, papa.
+narrateur|Papa pose un doigt, avec lui.
+narrateur|Maman pose un doigt, aussi.
+enfant-m|Vous touchez.
+maman|Il est froid, près de l'eau ?
+enfant-m|Un peu.
+narrateur|Le galet sent l'herbe tiède.
+narrateur|Une petite trace d'eau reste.
+enfant-m|Poumf.
+papa|Le galet tient, Victorino ?
+enfant-m|Oui, papa.
+maman|Tes genoux sont au chaud ?
+enfant-m|Un peu, maman.
+narrateur|La nappe reste ouverte, près d'eux.
+enfant-m|Elle sent le pain.
+papa|On reste ici, Victorino ?
+enfant-m|Oui.
+narrateur|Les cailloux font tic, au bord.
+enfant-m|Le tic est là.
+maman|Tu le serres sans forcer ?
 enfant-m|Oui, maman.
-papa|Tu as bien invité.
-enfant-m|Je suis content.
-maman|La joie est là, près de l'eau.
-narrateur|Ils s'assoient sur la nappe.
-maman|Tu as les pieds dans l'herbe ?
-enfant-m|Oui. Dans l'herbe.
-narrateur|Le pain attend dans le panier.
-narrateur|L'eau chante encore.
-papa|On goûte le pain après ?
-enfant-m|Après. Le galet d'abord.</t>
+papa|On touche ensemble ?
+enfant-m|Oui.
+narrateur|Trois doigts tiennent le galet.
+enfant-m|Il ne part plus.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>eau</t>
         </is>
       </c>
     </row>
@@ -1941,17 +2052,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis content. On a partagé le galet. Bravo, Victorino.</t>
+          <t>Ils restent près de la nappe. Maman essuie un peu d'eau. Le galet a glissé, papa. Tu l'as vu, toi ? Oui, vers l'eau. On est bien, ici. Victorino tapote le galet du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le galet est resté, Victorino. Oui, dans ma main. Ça sent l'herbe, un peu tiède. Et le pain, maman. Oui, dans l'air. On reste au bord, Victorino ? Oui, papa. Le galet reste près de la nappe. Un éclat de berge tient près du bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis content. On a partagé le galet. Bravo, Victorino.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la nappe. Maman essuie un peu d'eau. Le galet a glissé, papa. Tu l'as vu, toi ? Oui, vers l'eau. On est bien, ici. Victorino tapote le galet du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le galet est resté, Victorino. Oui, dans ma main. Ça sent l'herbe, un peu tiède. Et le pain, maman. Oui, dans l'air. On reste au bord, Victorino ? Oui, papa. Le galet reste près de la nappe. Un &lt;emphasis level="moderate"&gt;éclat de berge&lt;/emphasis&gt; tient près du bord.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la nappe. Maman essuie un peu d'eau. Le galet a glissé, papa. Tu l'as vu, toi ? Oui, vers l'eau. On est bien, ici. Victorino tapote le galet du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le galet est resté, Victorino. Oui, dans ma main. Ça sent l'herbe, un peu tiède. Et le pain, maman. Oui, dans l'air. On reste au bord, Victorino ? Oui, papa. Le galet reste près de la nappe. Un &lt;emphasis&gt;éclat de berge&lt;/emphasis&gt; tient près du bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1998,7 +2109,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2006,7 +2117,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2018,12 +2129,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2032,14 +2143,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de berge</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2051,11 +2166,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2064,26 +2179,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pres_du_bord; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis content.
-enfant-m|On a partagé le galet.
-papa|Bravo, Victorino.</t>
+          <t>narrateur|Ils restent près de la nappe.
+narrateur|Maman essuie un peu d'eau.
+enfant-m|Le galet a glissé, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, vers l'eau.
+maman|On est bien, ici.
+narrateur|Victorino tapote le galet du doigt.
+enfant-m|Il a une trace d'eau.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le galet est resté, Victorino.
+enfant-m|Oui, dans ma main.
+narrateur|Ça sent l'herbe, un peu tiède.
+enfant-m|Et le pain, maman.
+maman|Oui, dans l'air.
+papa|On reste au bord, Victorino ?
+enfant-m|Oui, papa.
+narrateur|Le galet reste près de la nappe.
+narrateur|Un éclat de berge tient près du bord.</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2168,6 +2303,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>